<commit_message>
why did it take me so long to make one figure :,(
</commit_message>
<xml_diff>
--- a/EPFU_2025/EPFU 2025 Bleeding.xlsx
+++ b/EPFU_2025/EPFU 2025 Bleeding.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Ashlyn_thesis\EPFU_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24F335BC-6D4E-4DF3-BF7B-14F39082AE41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B723B00-76B6-4603-B432-3A737D759798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,7 +572,7 @@
     <numFmt numFmtId="164" formatCode="h&quot;:&quot;mm"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="[h]:mm"/>
-    <numFmt numFmtId="168" formatCode="h:mm;@"/>
+    <numFmt numFmtId="167" formatCode="h:mm;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -626,9 +626,9 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2710,7 +2710,7 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="N40" s="8">
-        <f>M40-D40</f>
+        <f t="shared" ref="N40:N71" si="0">M40-D40</f>
         <v>0.21388888888888891</v>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="N41" s="8">
-        <f>M41-D41</f>
+        <f t="shared" si="0"/>
         <v>0.21458333333333335</v>
       </c>
     </row>
@@ -2800,7 +2800,7 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="N42" s="8">
-        <f>M42-D42</f>
+        <f t="shared" si="0"/>
         <v>0.21597222222222223</v>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="N43" s="8" t="e">
-        <f>M43-D43</f>
+        <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
       <c r="O43" s="1" t="s">
@@ -2893,7 +2893,7 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="N44" s="8" t="e">
-        <f>M44-D44</f>
+        <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
       <c r="O44" s="1" t="s">
@@ -2941,7 +2941,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N45" s="8">
-        <f>M45-D45</f>
+        <f t="shared" si="0"/>
         <v>0.11180555555555549</v>
       </c>
     </row>
@@ -2986,7 +2986,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N46" s="8">
-        <f>M46-D46</f>
+        <f t="shared" si="0"/>
         <v>0.11249999999999993</v>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N47" s="8">
-        <f>M47-D47</f>
+        <f t="shared" si="0"/>
         <v>0.11388888888888882</v>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N48" s="8">
-        <f>M48-D48</f>
+        <f t="shared" si="0"/>
         <v>0.11388888888888882</v>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N49" s="8">
-        <f>M49-D49</f>
+        <f t="shared" si="0"/>
         <v>0.11458333333333326</v>
       </c>
       <c r="O49" s="1" t="s">
@@ -3169,7 +3169,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N50" s="8">
-        <f>M50-D50</f>
+        <f t="shared" si="0"/>
         <v>0.1152777777777777</v>
       </c>
       <c r="O50" s="1" t="s">
@@ -3217,7 +3217,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N51" s="8">
-        <f>M51-D51</f>
+        <f t="shared" si="0"/>
         <v>0.1152777777777777</v>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N52" s="8">
-        <f>M52-D52</f>
+        <f t="shared" si="0"/>
         <v>0.11597222222222214</v>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N53" s="8">
-        <f>M53-D53</f>
+        <f t="shared" si="0"/>
         <v>0.11597222222222214</v>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N54" s="8">
-        <f>M54-D54</f>
+        <f t="shared" si="0"/>
         <v>0.11597222222222214</v>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N55" s="8">
-        <f>M55-D55</f>
+        <f t="shared" si="0"/>
         <v>0.11666666666666659</v>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N56" s="8">
-        <f>M56-D56</f>
+        <f t="shared" si="0"/>
         <v>0.11666666666666659</v>
       </c>
     </row>
@@ -3487,7 +3487,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N57" s="8">
-        <f>M57-D57</f>
+        <f t="shared" si="0"/>
         <v>0.11736111111111103</v>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N58" s="8">
-        <f>M58-D58</f>
+        <f t="shared" si="0"/>
         <v>0.11805555555555547</v>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N59" s="8">
-        <f>M59-D59</f>
+        <f t="shared" si="0"/>
         <v>0.11805555555555547</v>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N60" s="8">
-        <f>M60-D60</f>
+        <f t="shared" si="0"/>
         <v>0.11874999999999991</v>
       </c>
       <c r="O60" s="1" t="s">
@@ -3670,7 +3670,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N61" s="8">
-        <f>M61-D61</f>
+        <f t="shared" si="0"/>
         <v>0.12847222222222221</v>
       </c>
     </row>
@@ -3715,7 +3715,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N62" s="8">
-        <f>M62-D62</f>
+        <f t="shared" si="0"/>
         <v>0.12916666666666665</v>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N63" s="8">
-        <f>M63-D63</f>
+        <f t="shared" si="0"/>
         <v>0.12916666666666665</v>
       </c>
     </row>
@@ -3805,7 +3805,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N64" s="8">
-        <f>M64-D64</f>
+        <f t="shared" si="0"/>
         <v>0.12916666666666665</v>
       </c>
       <c r="O64" s="1" t="s">
@@ -3853,7 +3853,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N65" s="8">
-        <f>M65-D65</f>
+        <f t="shared" si="0"/>
         <v>0.12916666666666665</v>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
         <v>0.62152777777777779</v>
       </c>
       <c r="H66" s="3">
-        <v>25.3</v>
+        <v>29.7</v>
       </c>
       <c r="I66" s="1" t="s">
         <v>18</v>
@@ -3898,7 +3898,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N66" s="8">
-        <f>M66-D66</f>
+        <f t="shared" si="0"/>
         <v>0.12986111111111109</v>
       </c>
     </row>
@@ -3943,7 +3943,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N67" s="8">
-        <f>M67-D67</f>
+        <f t="shared" si="0"/>
         <v>0.12986111111111109</v>
       </c>
       <c r="O67" s="1" t="s">
@@ -3991,7 +3991,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N68" s="8">
-        <f>M68-D68</f>
+        <f t="shared" si="0"/>
         <v>0.13055555555555554</v>
       </c>
     </row>
@@ -4036,7 +4036,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N69" s="8">
-        <f>M69-D69</f>
+        <f t="shared" si="0"/>
         <v>0.13055555555555554</v>
       </c>
     </row>
@@ -4081,7 +4081,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N70" s="8">
-        <f>M70-D70</f>
+        <f t="shared" si="0"/>
         <v>0.13055555555555554</v>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N71" s="8">
-        <f>M71-D71</f>
+        <f t="shared" si="0"/>
         <v>0.13055555555555554</v>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N72" s="8">
-        <f>M72-D72</f>
+        <f t="shared" ref="N72:N103" si="1">M72-D72</f>
         <v>0.13124999999999998</v>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N73" s="8">
-        <f>M73-D73</f>
+        <f t="shared" si="1"/>
         <v>0.13124999999999998</v>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N74" s="8">
-        <f>M74-D74</f>
+        <f t="shared" si="1"/>
         <v>0.13124999999999998</v>
       </c>
     </row>
@@ -4306,7 +4306,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N75" s="8">
-        <f>M75-D75</f>
+        <f t="shared" si="1"/>
         <v>0.13263888888888886</v>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N76" s="8">
-        <f>M76-D76</f>
+        <f t="shared" si="1"/>
         <v>0.13402777777777775</v>
       </c>
     </row>
@@ -4396,7 +4396,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N77" s="8">
-        <f>M77-D77</f>
+        <f t="shared" si="1"/>
         <v>0.13472222222222219</v>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N78" s="8">
-        <f>M78-D78</f>
+        <f t="shared" si="1"/>
         <v>0.13611111111111107</v>
       </c>
     </row>
@@ -4486,7 +4486,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N79" s="8">
-        <f>M79-D79</f>
+        <f t="shared" si="1"/>
         <v>0.13611111111111107</v>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N80" s="8">
-        <f>M80-D80</f>
+        <f t="shared" si="1"/>
         <v>0.13680555555555551</v>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N81" s="8">
-        <f>M81-D81</f>
+        <f t="shared" si="1"/>
         <v>0.13749999999999996</v>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N82" s="8">
-        <f>M82-D82</f>
+        <f t="shared" si="1"/>
         <v>0.1381944444444444</v>
       </c>
     </row>
@@ -4666,7 +4666,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N83" s="8">
-        <f>M83-D83</f>
+        <f t="shared" si="1"/>
         <v>0.14027777777777772</v>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N84" s="8">
-        <f>M84-D84</f>
+        <f t="shared" si="1"/>
         <v>0.14027777777777772</v>
       </c>
       <c r="O84" s="1" t="s">
@@ -4759,7 +4759,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N85" s="8">
-        <f>M85-D85</f>
+        <f t="shared" si="1"/>
         <v>0.14027777777777772</v>
       </c>
     </row>
@@ -4804,7 +4804,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N86" s="8">
-        <f>M86-D86</f>
+        <f t="shared" si="1"/>
         <v>0.14166666666666661</v>
       </c>
     </row>
@@ -4849,7 +4849,7 @@
         <v>0.7006944444444444</v>
       </c>
       <c r="N87" s="8">
-        <f>M87-D87</f>
+        <f t="shared" si="1"/>
         <v>0.14236111111111105</v>
       </c>
       <c r="O87" s="1" t="s">
@@ -4873,7 +4873,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N88" s="9">
-        <f>M88-D88</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O88" t="s">
@@ -4897,7 +4897,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N89" s="9">
-        <f>M89-D89</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O89" t="s">
@@ -4921,7 +4921,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N90" s="9">
-        <f>M90-D90</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O90" t="s">
@@ -4945,7 +4945,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N91" s="9">
-        <f>M91-D91</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O91" t="s">
@@ -4969,7 +4969,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N92" s="9">
-        <f>M92-D92</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O92" t="s">
@@ -4993,7 +4993,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N93" s="9">
-        <f>M93-D93</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O93" t="s">
@@ -5017,7 +5017,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N94" s="9">
-        <f>M94-D94</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O94" t="s">
@@ -5041,7 +5041,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N95" s="9">
-        <f>M95-D95</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O95" t="s">
@@ -5065,7 +5065,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N96" s="9">
-        <f>M96-D96</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O96" t="s">
@@ -5089,7 +5089,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N97" s="9">
-        <f>M97-D97</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O97" t="s">
@@ -5113,7 +5113,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N98" s="9">
-        <f>M98-D98</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O98" t="s">
@@ -5137,7 +5137,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N99" s="9">
-        <f>M99-D99</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O99" t="s">
@@ -5161,7 +5161,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N100" s="9">
-        <f>M100-D100</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O100" t="s">
@@ -5185,7 +5185,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N101" s="9">
-        <f>M101-D101</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O101" t="s">
@@ -5209,7 +5209,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N102" s="9">
-        <f>M102-D102</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O102" t="s">
@@ -5233,7 +5233,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N103" s="9">
-        <f>M103-D103</f>
+        <f t="shared" si="1"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O103" t="s">
@@ -5257,7 +5257,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N104" s="9">
-        <f>M104-D104</f>
+        <f t="shared" ref="N104:N135" si="2">M104-D104</f>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O104" t="s">
@@ -5281,7 +5281,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N105" s="9">
-        <f>M105-D105</f>
+        <f t="shared" si="2"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O105" t="s">
@@ -5305,7 +5305,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N106" s="9">
-        <f>M106-D106</f>
+        <f t="shared" si="2"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O106" t="s">
@@ -5329,7 +5329,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N107" s="9">
-        <f>M107-D107</f>
+        <f t="shared" si="2"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O107" t="s">
@@ -5353,7 +5353,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N108" s="9">
-        <f>M108-D108</f>
+        <f t="shared" si="2"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O108" t="s">
@@ -5377,7 +5377,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N109" s="9">
-        <f>M109-D109</f>
+        <f t="shared" si="2"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O109" t="s">
@@ -5401,7 +5401,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="N110" s="9">
-        <f>M110-D110</f>
+        <f t="shared" si="2"/>
         <v>1.7361111111111049E-2</v>
       </c>
       <c r="O110" t="s">
@@ -5449,7 +5449,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N111" s="8">
-        <f>M111-D111</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O111" s="1" t="s">
@@ -5498,7 +5498,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N112" s="8">
-        <f>M112-D112</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O112" s="1" t="s">
@@ -5547,7 +5547,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N113" s="8">
-        <f>M113-D113</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O113" s="1" t="s">
@@ -5596,7 +5596,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N114" s="8">
-        <f>M114-D114</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O114" s="1" t="s">
@@ -5645,7 +5645,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N115" s="8">
-        <f>M115-D115</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O115" s="1" t="s">
@@ -5694,7 +5694,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N116" s="8">
-        <f>M116-D116</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O116" s="1" t="s">
@@ -5743,7 +5743,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N117" s="8">
-        <f>M117-D117</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O117" s="1" t="s">
@@ -5792,7 +5792,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N118" s="8">
-        <f>M118-D118</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O118" s="1" t="s">
@@ -5841,7 +5841,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N119" s="8">
-        <f>M119-D119</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O119" s="1" t="s">
@@ -5890,7 +5890,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N120" s="8">
-        <f>M120-D120</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O120" s="1" t="s">
@@ -5939,7 +5939,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N121" s="8">
-        <f>M121-D121</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O121" s="1" t="s">
@@ -5988,7 +5988,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N122" s="8">
-        <f>M122-D122</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O122" s="1" t="s">
@@ -6037,7 +6037,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N123" s="8">
-        <f>M123-D123</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O123" s="1" t="s">
@@ -6086,7 +6086,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N124" s="8">
-        <f>M124-D124</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O124" s="1" t="s">
@@ -6135,7 +6135,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N125" s="8">
-        <f>M125-D125</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O125" s="1" t="s">
@@ -6184,7 +6184,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N126" s="8">
-        <f>M126-D126</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O126" s="1" t="s">
@@ -6233,7 +6233,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N127" s="8">
-        <f>M127-D127</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O127" s="1" t="s">
@@ -6282,7 +6282,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="N128" s="8">
-        <f>M128-D128</f>
+        <f t="shared" si="2"/>
         <v>9.8611111111111094E-2</v>
       </c>
       <c r="O128" s="1" t="s">
@@ -6331,7 +6331,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N129" s="8">
-        <f>M129-D129</f>
+        <f t="shared" si="2"/>
         <v>0.11874999999999991</v>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N130" s="8">
-        <f>M130-D130</f>
+        <f t="shared" si="2"/>
         <v>0.11874999999999991</v>
       </c>
     </row>
@@ -6421,7 +6421,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N131" s="8">
-        <f>M131-D131</f>
+        <f t="shared" si="2"/>
         <v>0.11874999999999991</v>
       </c>
     </row>
@@ -6466,7 +6466,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N132" s="8">
-        <f>M132-D132</f>
+        <f t="shared" si="2"/>
         <v>0.11944444444444435</v>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N133" s="8">
-        <f>M133-D133</f>
+        <f t="shared" si="2"/>
         <v>0.11944444444444435</v>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N134" s="8">
-        <f>M134-D134</f>
+        <f t="shared" si="2"/>
         <v>0.12013888888888891</v>
       </c>
     </row>
@@ -6601,7 +6601,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N135" s="8">
-        <f>M135-D135</f>
+        <f t="shared" si="2"/>
         <v>0.12013888888888891</v>
       </c>
     </row>
@@ -6646,7 +6646,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N136" s="8">
-        <f>M136-D136</f>
+        <f t="shared" ref="N136:N167" si="3">M136-D136</f>
         <v>0.12083333333333335</v>
       </c>
     </row>
@@ -6691,7 +6691,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N137" s="8">
-        <f>M137-D137</f>
+        <f t="shared" si="3"/>
         <v>0.12083333333333335</v>
       </c>
     </row>
@@ -6736,7 +6736,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N138" s="8">
-        <f>M138-D138</f>
+        <f t="shared" si="3"/>
         <v>0.12083333333333335</v>
       </c>
     </row>
@@ -6781,7 +6781,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N139" s="8">
-        <f>M139-D139</f>
+        <f t="shared" si="3"/>
         <v>0.12152777777777779</v>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N140" s="8">
-        <f>M140-D140</f>
+        <f t="shared" si="3"/>
         <v>0.12152777777777779</v>
       </c>
     </row>
@@ -6871,7 +6871,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N141" s="8">
-        <f>M141-D141</f>
+        <f t="shared" si="3"/>
         <v>0.12222222222222223</v>
       </c>
     </row>
@@ -6916,7 +6916,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N142" s="8">
-        <f>M142-D142</f>
+        <f t="shared" si="3"/>
         <v>0.12222222222222223</v>
       </c>
     </row>
@@ -6961,7 +6961,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N143" s="8">
-        <f>M143-D143</f>
+        <f t="shared" si="3"/>
         <v>0.12291666666666667</v>
       </c>
     </row>
@@ -7006,7 +7006,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N144" s="8">
-        <f>M144-D144</f>
+        <f t="shared" si="3"/>
         <v>0.125</v>
       </c>
     </row>
@@ -7051,7 +7051,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N145" s="8">
-        <f>M145-D145</f>
+        <f t="shared" si="3"/>
         <v>0.12569444444444444</v>
       </c>
     </row>
@@ -7096,7 +7096,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N146" s="8">
-        <f>M146-D146</f>
+        <f t="shared" si="3"/>
         <v>0.12638888888888888</v>
       </c>
     </row>
@@ -7141,7 +7141,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N147" s="8">
-        <f>M147-D147</f>
+        <f t="shared" si="3"/>
         <v>0.12708333333333333</v>
       </c>
     </row>
@@ -7186,7 +7186,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N148" s="8">
-        <f>M148-D148</f>
+        <f t="shared" si="3"/>
         <v>0.12708333333333333</v>
       </c>
     </row>
@@ -7231,7 +7231,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N149" s="8">
-        <f>M149-D149</f>
+        <f t="shared" si="3"/>
         <v>0.12777777777777777</v>
       </c>
     </row>
@@ -7276,7 +7276,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N150" s="8">
-        <f>M150-D150</f>
+        <f t="shared" si="3"/>
         <v>0.12777777777777777</v>
       </c>
     </row>
@@ -7321,7 +7321,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N151" s="8">
-        <f>M151-D151</f>
+        <f t="shared" si="3"/>
         <v>0.12777777777777777</v>
       </c>
     </row>
@@ -7342,7 +7342,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N152" s="8">
-        <f>M152-D152</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O152" t="s">
@@ -7366,7 +7366,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N153" s="8">
-        <f>M153-D153</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O153" t="s">
@@ -7390,7 +7390,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N154" s="8">
-        <f>M154-D154</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O154" t="s">
@@ -7414,7 +7414,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N155" s="8">
-        <f>M155-D155</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O155" t="s">
@@ -7438,7 +7438,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N156" s="8">
-        <f>M156-D156</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O156" t="s">
@@ -7462,7 +7462,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N157" s="8">
-        <f>M157-D157</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O157" t="s">
@@ -7486,7 +7486,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N158" s="8">
-        <f>M158-D158</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O158" t="s">
@@ -7510,7 +7510,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N159" s="8">
-        <f>M159-D159</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O159" t="s">
@@ -7534,7 +7534,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N160" s="8">
-        <f>M160-D160</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O160" t="s">
@@ -7558,7 +7558,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N161" s="8">
-        <f>M161-D161</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O161" t="s">
@@ -7582,7 +7582,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N162" s="8">
-        <f>M162-D162</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O162" t="s">
@@ -7606,7 +7606,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N163" s="8">
-        <f>M163-D163</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O163" t="s">
@@ -7630,7 +7630,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N164" s="8">
-        <f>M164-D164</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O164" t="s">
@@ -7654,7 +7654,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N165" s="8">
-        <f>M165-D165</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O165" t="s">
@@ -7678,7 +7678,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N166" s="8">
-        <f>M166-D166</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O166" t="s">
@@ -7702,7 +7702,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N167" s="8">
-        <f>M167-D167</f>
+        <f t="shared" si="3"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O167" t="s">
@@ -7726,7 +7726,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N168" s="8">
-        <f>M168-D168</f>
+        <f t="shared" ref="N168:N199" si="4">M168-D168</f>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O168" t="s">
@@ -7750,7 +7750,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N169" s="8">
-        <f>M169-D169</f>
+        <f t="shared" si="4"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O169" t="s">
@@ -7774,7 +7774,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N170" s="8">
-        <f>M170-D170</f>
+        <f t="shared" si="4"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O170" t="s">
@@ -7798,7 +7798,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N171" s="8">
-        <f>M171-D171</f>
+        <f t="shared" si="4"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O171" t="s">
@@ -7822,7 +7822,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N172" s="8">
-        <f>M172-D172</f>
+        <f t="shared" si="4"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O172" t="s">
@@ -7846,7 +7846,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N173" s="8">
-        <f>M173-D173</f>
+        <f t="shared" si="4"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O173" t="s">
@@ -7870,7 +7870,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N174" s="8">
-        <f>M174-D174</f>
+        <f t="shared" si="4"/>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O174" t="s">
@@ -9328,7 +9328,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N205" s="8">
-        <f>M205-D205</f>
+        <f t="shared" ref="N205:N236" si="5">M205-D205</f>
         <v>0.18819444444444444</v>
       </c>
       <c r="O205" s="1" t="s">
@@ -9376,7 +9376,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N206" s="8">
-        <f>M206-D206</f>
+        <f t="shared" si="5"/>
         <v>0.18888888888888888</v>
       </c>
     </row>
@@ -9421,7 +9421,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N207" s="8">
-        <f>M207-D207</f>
+        <f t="shared" si="5"/>
         <v>6.3888888888888884E-2</v>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N208" s="8">
-        <f>M208-D208</f>
+        <f t="shared" si="5"/>
         <v>6.3888888888888884E-2</v>
       </c>
     </row>
@@ -9511,7 +9511,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N209" s="8">
-        <f>M209-D209</f>
+        <f t="shared" si="5"/>
         <v>6.4583333333333326E-2</v>
       </c>
     </row>
@@ -9556,7 +9556,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N210" s="8">
-        <f>M210-D210</f>
+        <f t="shared" si="5"/>
         <v>6.4583333333333326E-2</v>
       </c>
       <c r="O210" s="1" t="s">
@@ -9604,7 +9604,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N211" s="8">
-        <f>M211-D211</f>
+        <f t="shared" si="5"/>
         <v>6.5277777777777768E-2</v>
       </c>
     </row>
@@ -9649,7 +9649,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N212" s="8">
-        <f>M212-D212</f>
+        <f t="shared" si="5"/>
         <v>7.638888888888884E-2</v>
       </c>
       <c r="O212" s="1" t="s">
@@ -9697,7 +9697,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N213" s="8">
-        <f>M213-D213</f>
+        <f t="shared" si="5"/>
         <v>7.7083333333333282E-2</v>
       </c>
       <c r="O213" s="1" t="s">
@@ -9745,7 +9745,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N214" s="8">
-        <f>M214-D214</f>
+        <f t="shared" si="5"/>
         <v>7.7777777777777724E-2</v>
       </c>
     </row>
@@ -9790,7 +9790,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N215" s="8">
-        <f>M215-D215</f>
+        <f t="shared" si="5"/>
         <v>7.8472222222222165E-2</v>
       </c>
     </row>
@@ -9835,7 +9835,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N216" s="8">
-        <f>M216-D216</f>
+        <f t="shared" si="5"/>
         <v>7.9166666666666607E-2</v>
       </c>
     </row>
@@ -9880,7 +9880,7 @@
         <v>0.63055555555555554</v>
       </c>
       <c r="N217" s="8">
-        <f>M217-D217</f>
+        <f t="shared" si="5"/>
         <v>7.9861111111111049E-2</v>
       </c>
     </row>
@@ -9925,7 +9925,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N218" s="8">
-        <f>M218-D218</f>
+        <f t="shared" si="5"/>
         <v>0.12777777777777777</v>
       </c>
     </row>
@@ -9970,7 +9970,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N219" s="8">
-        <f>M219-D219</f>
+        <f t="shared" si="5"/>
         <v>0.12777777777777777</v>
       </c>
     </row>
@@ -10015,7 +10015,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N220" s="8">
-        <f>M220-D220</f>
+        <f t="shared" si="5"/>
         <v>0.12777777777777777</v>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N221" s="8">
-        <f>M221-D221</f>
+        <f t="shared" si="5"/>
         <v>0.12986111111111109</v>
       </c>
     </row>
@@ -10105,7 +10105,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N222" s="8">
-        <f>M222-D222</f>
+        <f t="shared" si="5"/>
         <v>0.12986111111111109</v>
       </c>
     </row>
@@ -10150,7 +10150,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N223" s="8">
-        <f>M223-D223</f>
+        <f t="shared" si="5"/>
         <v>0.12986111111111109</v>
       </c>
     </row>
@@ -10195,7 +10195,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N224" s="8">
-        <f>M224-D224</f>
+        <f t="shared" si="5"/>
         <v>0.12986111111111109</v>
       </c>
     </row>
@@ -10240,7 +10240,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N225" s="8">
-        <f>M225-D225</f>
+        <f t="shared" si="5"/>
         <v>0.1381944444444444</v>
       </c>
     </row>
@@ -10285,7 +10285,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N226" s="8">
-        <f>M226-D226</f>
+        <f t="shared" si="5"/>
         <v>0.1381944444444444</v>
       </c>
     </row>
@@ -10330,7 +10330,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N227" s="8">
-        <f>M227-D227</f>
+        <f t="shared" si="5"/>
         <v>0.14236111111111105</v>
       </c>
     </row>
@@ -10375,7 +10375,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N228" s="8">
-        <f>M228-D228</f>
+        <f t="shared" si="5"/>
         <v>0.14305555555555549</v>
       </c>
     </row>
@@ -10402,7 +10402,7 @@
         <v>0.65</v>
       </c>
       <c r="H229" s="3">
-        <v>24.4</v>
+        <v>30.5</v>
       </c>
       <c r="I229" s="1" t="s">
         <v>18</v>
@@ -10420,7 +10420,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N229" s="8">
-        <f>M229-D229</f>
+        <f t="shared" si="5"/>
         <v>0.14305555555555549</v>
       </c>
     </row>
@@ -10465,7 +10465,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N230" s="8">
-        <f>M230-D230</f>
+        <f t="shared" si="5"/>
         <v>0.14305555555555549</v>
       </c>
     </row>
@@ -10510,7 +10510,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N231" s="8">
-        <f>M231-D231</f>
+        <f t="shared" si="5"/>
         <v>0.14374999999999993</v>
       </c>
     </row>
@@ -10555,7 +10555,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N232" s="8">
-        <f>M232-D232</f>
+        <f t="shared" si="5"/>
         <v>0.14444444444444438</v>
       </c>
       <c r="O232" s="1" t="s">
@@ -10603,7 +10603,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N233" s="8">
-        <f>M233-D233</f>
+        <f t="shared" si="5"/>
         <v>0.14444444444444438</v>
       </c>
     </row>
@@ -10648,7 +10648,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N234" s="8">
-        <f>M234-D234</f>
+        <f t="shared" si="5"/>
         <v>0.14444444444444438</v>
       </c>
       <c r="O234" s="1" t="s">
@@ -10696,7 +10696,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N235" s="8">
-        <f>M235-D235</f>
+        <f t="shared" si="5"/>
         <v>0.14444444444444438</v>
       </c>
     </row>
@@ -10741,7 +10741,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N236" s="8">
-        <f>M236-D236</f>
+        <f t="shared" si="5"/>
         <v>0.14513888888888882</v>
       </c>
     </row>
@@ -10786,7 +10786,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="N237" s="8">
-        <f>M237-D237</f>
+        <f t="shared" ref="N237:N268" si="6">M237-D237</f>
         <v>0.14513888888888882</v>
       </c>
     </row>
@@ -10831,7 +10831,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N238" s="8">
-        <f>M238-D238</f>
+        <f t="shared" si="6"/>
         <v>5.2777777777777701E-2</v>
       </c>
     </row>
@@ -10876,7 +10876,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N239" s="8">
-        <f>M239-D239</f>
+        <f t="shared" si="6"/>
         <v>5.4166666666666585E-2</v>
       </c>
     </row>
@@ -10921,7 +10921,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N240" s="8">
-        <f>M240-D240</f>
+        <f t="shared" si="6"/>
         <v>5.4166666666666585E-2</v>
       </c>
     </row>
@@ -10966,7 +10966,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N241" s="8">
-        <f>M241-D241</f>
+        <f t="shared" si="6"/>
         <v>5.4166666666666585E-2</v>
       </c>
     </row>
@@ -11011,7 +11011,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N242" s="8">
-        <f>M242-D242</f>
+        <f t="shared" si="6"/>
         <v>5.4166666666666585E-2</v>
       </c>
     </row>
@@ -11056,7 +11056,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N243" s="8">
-        <f>M243-D243</f>
+        <f t="shared" si="6"/>
         <v>5.4861111111111027E-2</v>
       </c>
     </row>
@@ -11101,7 +11101,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N244" s="8">
-        <f>M244-D244</f>
+        <f t="shared" si="6"/>
         <v>5.4861111111111027E-2</v>
       </c>
     </row>
@@ -11146,7 +11146,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N245" s="8">
-        <f>M245-D245</f>
+        <f t="shared" si="6"/>
         <v>5.5555555555555469E-2</v>
       </c>
     </row>
@@ -11191,7 +11191,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N246" s="8">
-        <f>M246-D246</f>
+        <f t="shared" si="6"/>
         <v>5.5555555555555469E-2</v>
       </c>
     </row>
@@ -11236,7 +11236,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N247" s="8">
-        <f>M247-D247</f>
+        <f t="shared" si="6"/>
         <v>5.6249999999999911E-2</v>
       </c>
     </row>
@@ -11281,7 +11281,7 @@
         <v>0.60624999999999996</v>
       </c>
       <c r="N248" s="8">
-        <f>M248-D248</f>
+        <f t="shared" si="6"/>
         <v>5.6249999999999911E-2</v>
       </c>
     </row>
@@ -11326,7 +11326,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N249" s="8">
-        <f>M249-D249</f>
+        <f t="shared" si="6"/>
         <v>0.11319444444444438</v>
       </c>
     </row>
@@ -11371,7 +11371,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N250" s="8">
-        <f>M250-D250</f>
+        <f t="shared" si="6"/>
         <v>0.11319444444444438</v>
       </c>
     </row>
@@ -11416,7 +11416,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N251" s="8">
-        <f>M251-D251</f>
+        <f t="shared" si="6"/>
         <v>0.11319444444444438</v>
       </c>
     </row>
@@ -11461,7 +11461,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N252" s="8">
-        <f>M252-D252</f>
+        <f t="shared" si="6"/>
         <v>0.11388888888888882</v>
       </c>
     </row>
@@ -11506,7 +11506,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N253" s="8">
-        <f>M253-D253</f>
+        <f t="shared" si="6"/>
         <v>0.11458333333333326</v>
       </c>
     </row>
@@ -11551,7 +11551,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N254" s="8">
-        <f>M254-D254</f>
+        <f t="shared" si="6"/>
         <v>0.11458333333333326</v>
       </c>
     </row>
@@ -11596,7 +11596,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N255" s="8">
-        <f>M255-D255</f>
+        <f t="shared" si="6"/>
         <v>0.11458333333333326</v>
       </c>
     </row>
@@ -11641,7 +11641,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N256" s="8">
-        <f>M256-D256</f>
+        <f t="shared" si="6"/>
         <v>0.11458333333333326</v>
       </c>
     </row>
@@ -11686,7 +11686,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N257" s="8">
-        <f>M257-D257</f>
+        <f t="shared" si="6"/>
         <v>0.1152777777777777</v>
       </c>
       <c r="O257" s="1" t="s">
@@ -11734,7 +11734,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N258" s="8">
-        <f>M258-D258</f>
+        <f t="shared" si="6"/>
         <v>0.1152777777777777</v>
       </c>
     </row>
@@ -11779,7 +11779,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N259" s="8">
-        <f>M259-D259</f>
+        <f t="shared" si="6"/>
         <v>0.1152777777777777</v>
       </c>
     </row>
@@ -11824,7 +11824,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N260" s="8">
-        <f>M260-D260</f>
+        <f t="shared" si="6"/>
         <v>0.1152777777777777</v>
       </c>
     </row>
@@ -11869,7 +11869,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N261" s="8">
-        <f>M261-D261</f>
+        <f t="shared" si="6"/>
         <v>0.11597222222222214</v>
       </c>
     </row>
@@ -11914,7 +11914,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N262" s="8">
-        <f>M262-D262</f>
+        <f t="shared" si="6"/>
         <v>0.11597222222222214</v>
       </c>
       <c r="O262" s="1" t="s">
@@ -11962,7 +11962,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N263" s="8">
-        <f>M263-D263</f>
+        <f t="shared" si="6"/>
         <v>0.11666666666666659</v>
       </c>
       <c r="O263" s="1" t="s">
@@ -12010,7 +12010,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N264" s="8">
-        <f>M264-D264</f>
+        <f t="shared" si="6"/>
         <v>0.11666666666666659</v>
       </c>
     </row>
@@ -12055,7 +12055,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N265" s="8">
-        <f>M265-D265</f>
+        <f t="shared" si="6"/>
         <v>0.11666666666666659</v>
       </c>
     </row>
@@ -12100,7 +12100,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N266" s="8">
-        <f>M266-D266</f>
+        <f t="shared" si="6"/>
         <v>0.11666666666666659</v>
       </c>
     </row>
@@ -12145,7 +12145,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="N267" s="8">
-        <f>M267-D267</f>
+        <f t="shared" si="6"/>
         <v>0.11736111111111103</v>
       </c>
     </row>
@@ -12190,7 +12190,7 @@
         <v>0.625</v>
       </c>
       <c r="N268" s="8">
-        <f>M268-D268</f>
+        <f t="shared" si="6"/>
         <v>6.3888888888888884E-2</v>
       </c>
       <c r="O268" s="1" t="s">
@@ -12238,7 +12238,7 @@
         <v>0.625</v>
       </c>
       <c r="N269" s="8">
-        <f>M269-D269</f>
+        <f t="shared" ref="N269:N300" si="7">M269-D269</f>
         <v>6.5277777777777768E-2</v>
       </c>
     </row>
@@ -12283,7 +12283,7 @@
         <v>0.625</v>
       </c>
       <c r="N270" s="8">
-        <f>M270-D270</f>
+        <f t="shared" si="7"/>
         <v>6.5277777777777768E-2</v>
       </c>
     </row>
@@ -12328,7 +12328,7 @@
         <v>0.625</v>
       </c>
       <c r="N271" s="8">
-        <f>M271-D271</f>
+        <f t="shared" si="7"/>
         <v>6.7361111111111094E-2</v>
       </c>
     </row>
@@ -12373,7 +12373,7 @@
         <v>0.625</v>
       </c>
       <c r="N272" s="8">
-        <f>M272-D272</f>
+        <f t="shared" si="7"/>
         <v>6.8749999999999978E-2</v>
       </c>
     </row>
@@ -12418,7 +12418,7 @@
         <v>0.625</v>
       </c>
       <c r="N273" s="8">
-        <f>M273-D273</f>
+        <f t="shared" si="7"/>
         <v>6.944444444444442E-2</v>
       </c>
     </row>
@@ -12463,7 +12463,7 @@
         <v>0.625</v>
       </c>
       <c r="N274" s="8">
-        <f>M274-D274</f>
+        <f t="shared" si="7"/>
         <v>6.944444444444442E-2</v>
       </c>
     </row>
@@ -12508,7 +12508,7 @@
         <v>0.625</v>
       </c>
       <c r="N275" s="8">
-        <f>M275-D275</f>
+        <f t="shared" si="7"/>
         <v>7.0138888888888862E-2</v>
       </c>
     </row>
@@ -12553,7 +12553,7 @@
         <v>0.625</v>
       </c>
       <c r="N276" s="8">
-        <f>M276-D276</f>
+        <f t="shared" si="7"/>
         <v>7.0138888888888862E-2</v>
       </c>
     </row>
@@ -12598,7 +12598,7 @@
         <v>0.625</v>
       </c>
       <c r="N277" s="8">
-        <f>M277-D277</f>
+        <f t="shared" si="7"/>
         <v>7.0138888888888862E-2</v>
       </c>
     </row>
@@ -12643,7 +12643,7 @@
         <v>0.625</v>
       </c>
       <c r="N278" s="8">
-        <f>M278-D278</f>
+        <f t="shared" si="7"/>
         <v>7.0138888888888862E-2</v>
       </c>
     </row>
@@ -12688,7 +12688,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N279" s="8">
-        <f>M279-D279</f>
+        <f t="shared" si="7"/>
         <v>0.11250000000000004</v>
       </c>
     </row>
@@ -12733,7 +12733,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N280" s="8">
-        <f>M280-D280</f>
+        <f t="shared" si="7"/>
         <v>0.11388888888888893</v>
       </c>
     </row>
@@ -12778,7 +12778,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N281" s="8">
-        <f>M281-D281</f>
+        <f t="shared" si="7"/>
         <v>0.11388888888888893</v>
       </c>
     </row>
@@ -12823,7 +12823,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N282" s="8">
-        <f>M282-D282</f>
+        <f t="shared" si="7"/>
         <v>0.11458333333333337</v>
       </c>
     </row>
@@ -12868,7 +12868,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N283" s="8">
-        <f>M283-D283</f>
+        <f t="shared" si="7"/>
         <v>0.11527777777777781</v>
       </c>
     </row>
@@ -12913,7 +12913,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N284" s="8">
-        <f>M284-D284</f>
+        <f t="shared" si="7"/>
         <v>0.11597222222222225</v>
       </c>
     </row>
@@ -12958,7 +12958,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N285" s="8">
-        <f>M285-D285</f>
+        <f t="shared" si="7"/>
         <v>0.1166666666666667</v>
       </c>
     </row>
@@ -13003,7 +13003,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N286" s="8">
-        <f>M286-D286</f>
+        <f t="shared" si="7"/>
         <v>0.11805555555555558</v>
       </c>
     </row>
@@ -13048,7 +13048,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N287" s="8">
-        <f>M287-D287</f>
+        <f t="shared" si="7"/>
         <v>0.11944444444444446</v>
       </c>
     </row>
@@ -13093,7 +13093,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N288" s="8">
-        <f>M288-D288</f>
+        <f t="shared" si="7"/>
         <v>0.12013888888888891</v>
       </c>
     </row>
@@ -13138,7 +13138,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N289" s="8">
-        <f>M289-D289</f>
+        <f t="shared" si="7"/>
         <v>0.12083333333333335</v>
       </c>
     </row>
@@ -13183,7 +13183,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N290" s="8">
-        <f>M290-D290</f>
+        <f t="shared" si="7"/>
         <v>0.12222222222222223</v>
       </c>
     </row>
@@ -13228,7 +13228,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N291" s="8">
-        <f>M291-D291</f>
+        <f t="shared" si="7"/>
         <v>0.12222222222222223</v>
       </c>
     </row>
@@ -13273,7 +13273,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N292" s="8">
-        <f>M292-D292</f>
+        <f t="shared" si="7"/>
         <v>0.12291666666666667</v>
       </c>
     </row>
@@ -13318,7 +13318,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N293" s="8">
-        <f>M293-D293</f>
+        <f t="shared" si="7"/>
         <v>0.12361111111111112</v>
       </c>
     </row>
@@ -13363,7 +13363,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N294" s="8">
-        <f>M294-D294</f>
+        <f t="shared" si="7"/>
         <v>0.12430555555555556</v>
       </c>
     </row>
@@ -13408,7 +13408,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N295" s="8">
-        <f>M295-D295</f>
+        <f t="shared" si="7"/>
         <v>0.12569444444444444</v>
       </c>
     </row>
@@ -13453,7 +13453,7 @@
         <v>0.79791666666666672</v>
       </c>
       <c r="N296" s="8">
-        <f>M296-D296</f>
+        <f t="shared" si="7"/>
         <v>0.12638888888888899</v>
       </c>
       <c r="O296" s="1" t="s">
@@ -13501,7 +13501,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N297" s="8">
-        <f>M297-D297</f>
+        <f t="shared" si="7"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13546,7 +13546,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N298" s="8">
-        <f>M298-D298</f>
+        <f t="shared" si="7"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13591,7 +13591,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N299" s="8">
-        <f>M299-D299</f>
+        <f t="shared" si="7"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13636,7 +13636,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N300" s="8">
-        <f>M300-D300</f>
+        <f t="shared" si="7"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13681,7 +13681,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N301" s="8">
-        <f>M301-D301</f>
+        <f t="shared" ref="N301:N332" si="8">M301-D301</f>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13726,7 +13726,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N302" s="8">
-        <f>M302-D302</f>
+        <f t="shared" si="8"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13771,7 +13771,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N303" s="8">
-        <f>M303-D303</f>
+        <f t="shared" si="8"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13816,7 +13816,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N304" s="8">
-        <f>M304-D304</f>
+        <f t="shared" si="8"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13861,7 +13861,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N305" s="8">
-        <f>M305-D305</f>
+        <f t="shared" si="8"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13906,7 +13906,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N306" s="8">
-        <f>M306-D306</f>
+        <f t="shared" si="8"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13951,7 +13951,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N307" s="8">
-        <f>M307-D307</f>
+        <f t="shared" si="8"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -13996,7 +13996,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N308" s="8">
-        <f>M308-D308</f>
+        <f t="shared" si="8"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -14017,7 +14017,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N309" s="8">
-        <f>M309-D309</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O309" t="s">
@@ -14041,7 +14041,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N310" s="8">
-        <f>M310-D310</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O310" t="s">
@@ -14065,7 +14065,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N311" s="8">
-        <f>M311-D311</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O311" t="s">
@@ -14089,7 +14089,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N312" s="8">
-        <f>M312-D312</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O312" t="s">
@@ -14113,7 +14113,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N313" s="8">
-        <f>M313-D313</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O313" t="s">
@@ -14137,7 +14137,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N314" s="8">
-        <f>M314-D314</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O314" t="s">
@@ -14161,7 +14161,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N315" s="8">
-        <f>M315-D315</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O315" t="s">
@@ -14185,7 +14185,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N316" s="8">
-        <f>M316-D316</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O316" t="s">
@@ -14209,7 +14209,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N317" s="8">
-        <f>M317-D317</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O317" t="s">
@@ -14233,7 +14233,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N318" s="8">
-        <f>M318-D318</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O318" t="s">
@@ -14257,7 +14257,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N319" s="8">
-        <f>M319-D319</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O319" t="s">
@@ -14281,7 +14281,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N320" s="8">
-        <f>M320-D320</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O320" t="s">
@@ -14305,7 +14305,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N321" s="8">
-        <f>M321-D321</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O321" t="s">
@@ -14329,7 +14329,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N322" s="8">
-        <f>M322-D322</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O322" t="s">
@@ -14353,7 +14353,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N323" s="8">
-        <f>M323-D323</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O323" t="s">
@@ -14377,7 +14377,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N324" s="8">
-        <f>M324-D324</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O324" t="s">
@@ -14401,7 +14401,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N325" s="8">
-        <f>M325-D325</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O325" t="s">
@@ -14425,7 +14425,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N326" s="8">
-        <f>M326-D326</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O326" t="s">
@@ -14449,7 +14449,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N327" s="8">
-        <f>M327-D327</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O327" t="s">
@@ -14473,7 +14473,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N328" s="8">
-        <f>M328-D328</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O328" t="s">
@@ -14497,7 +14497,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N329" s="8">
-        <f>M329-D329</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O329" t="s">
@@ -14521,7 +14521,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N330" s="8">
-        <f>M330-D330</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O330" t="s">
@@ -14545,7 +14545,7 @@
         <v>0.51180555555555551</v>
       </c>
       <c r="N331" s="8">
-        <f>M331-D331</f>
+        <f t="shared" si="8"/>
         <v>2.0138888888888873E-2</v>
       </c>
       <c r="O331" t="s">
@@ -14593,7 +14593,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N332" s="8">
-        <f>K332-D332</f>
+        <f t="shared" ref="N332:N343" si="9">K332-D332</f>
         <v>0.13402777777777775</v>
       </c>
     </row>
@@ -14638,7 +14638,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N333" s="8">
-        <f>K333-D333</f>
+        <f t="shared" si="9"/>
         <v>0.1381944444444444</v>
       </c>
     </row>
@@ -14683,7 +14683,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N334" s="8">
-        <f>K334-D334</f>
+        <f t="shared" si="9"/>
         <v>0.13888888888888884</v>
       </c>
       <c r="O334" s="1" t="s">
@@ -14731,7 +14731,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N335" s="8">
-        <f>K335-D335</f>
+        <f t="shared" si="9"/>
         <v>0.14027777777777772</v>
       </c>
     </row>
@@ -14776,7 +14776,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N336" s="8">
-        <f>K336-D336</f>
+        <f t="shared" si="9"/>
         <v>0.14027777777777772</v>
       </c>
     </row>
@@ -14821,7 +14821,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N337" s="8">
-        <f>K337-D337</f>
+        <f t="shared" si="9"/>
         <v>0.14166666666666661</v>
       </c>
     </row>
@@ -14866,7 +14866,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N338" s="8">
-        <f>K338-D338</f>
+        <f t="shared" si="9"/>
         <v>0.14374999999999993</v>
       </c>
       <c r="O338" s="1" t="s">
@@ -14914,7 +14914,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N339" s="8">
-        <f>K339-D339</f>
+        <f t="shared" si="9"/>
         <v>0.14374999999999993</v>
       </c>
     </row>
@@ -14959,7 +14959,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N340" s="8">
-        <f>K340-D340</f>
+        <f t="shared" si="9"/>
         <v>0.14444444444444438</v>
       </c>
     </row>
@@ -15004,7 +15004,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N341" s="8">
-        <f>K341-D341</f>
+        <f t="shared" si="9"/>
         <v>0.14583333333333326</v>
       </c>
     </row>
@@ -15049,7 +15049,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N342" s="8">
-        <f>K342-D342</f>
+        <f t="shared" si="9"/>
         <v>0.1465277777777777</v>
       </c>
     </row>
@@ -15094,7 +15094,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N343" s="8">
-        <f>K343-D343</f>
+        <f t="shared" si="9"/>
         <v>0.14722222222222214</v>
       </c>
     </row>
@@ -15139,7 +15139,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N344" s="8">
-        <f>M344-D344</f>
+        <f t="shared" ref="N344:N355" si="10">M344-D344</f>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15184,7 +15184,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N345" s="8">
-        <f>M345-D345</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15229,7 +15229,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N346" s="8">
-        <f>M346-D346</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15274,7 +15274,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N347" s="8">
-        <f>M347-D347</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15319,7 +15319,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N348" s="8">
-        <f>M348-D348</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15364,7 +15364,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N349" s="8">
-        <f>M349-D349</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15409,7 +15409,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N350" s="8">
-        <f>M350-D350</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15454,7 +15454,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N351" s="8">
-        <f>M351-D351</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15499,7 +15499,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N352" s="8">
-        <f>M352-D352</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15544,7 +15544,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N353" s="8">
-        <f>M353-D353</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15589,7 +15589,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N354" s="8">
-        <f>M354-D354</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N355" s="8">
-        <f>M355-D355</f>
+        <f t="shared" si="10"/>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -15679,7 +15679,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N356" s="8">
-        <f>K356-D356</f>
+        <f t="shared" ref="N356:N367" si="11">K356-D356</f>
         <v>0.13402777777777775</v>
       </c>
     </row>
@@ -15724,7 +15724,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N357" s="8">
-        <f>K357-D357</f>
+        <f t="shared" si="11"/>
         <v>0.13402777777777775</v>
       </c>
       <c r="O357" s="1" t="s">
@@ -15772,7 +15772,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N358" s="8">
-        <f>K358-D358</f>
+        <f t="shared" si="11"/>
         <v>0.13541666666666663</v>
       </c>
     </row>
@@ -15817,7 +15817,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N359" s="8">
-        <f>K359-D359</f>
+        <f t="shared" si="11"/>
         <v>0.13611111111111107</v>
       </c>
     </row>
@@ -15862,7 +15862,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N360" s="8">
-        <f>K360-D360</f>
+        <f t="shared" si="11"/>
         <v>0.13680555555555551</v>
       </c>
     </row>
@@ -15907,7 +15907,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N361" s="8">
-        <f>K361-D361</f>
+        <f t="shared" si="11"/>
         <v>0.13749999999999996</v>
       </c>
     </row>
@@ -15952,7 +15952,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N362" s="8">
-        <f>K362-D362</f>
+        <f t="shared" si="11"/>
         <v>0.14236111111111105</v>
       </c>
     </row>
@@ -15997,7 +15997,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N363" s="8">
-        <f>K363-D363</f>
+        <f t="shared" si="11"/>
         <v>0.14236111111111105</v>
       </c>
     </row>
@@ -16042,7 +16042,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N364" s="8">
-        <f>K364-D364</f>
+        <f t="shared" si="11"/>
         <v>0.14305555555555549</v>
       </c>
     </row>
@@ -16087,7 +16087,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N365" s="8">
-        <f>K365-D365</f>
+        <f t="shared" si="11"/>
         <v>0.14305555555555549</v>
       </c>
     </row>
@@ -16132,7 +16132,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N366" s="8">
-        <f>K366-D366</f>
+        <f t="shared" si="11"/>
         <v>0.14583333333333326</v>
       </c>
     </row>
@@ -16177,7 +16177,7 @@
         <v>0.6694444444444444</v>
       </c>
       <c r="N367" s="8">
-        <f>K367-D367</f>
+        <f t="shared" si="11"/>
         <v>0.15625</v>
       </c>
     </row>
@@ -16198,7 +16198,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N368" s="9">
-        <f>M368-D368</f>
+        <f t="shared" ref="N368:N399" si="12">M368-D368</f>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O368" t="s">
@@ -16222,7 +16222,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N369" s="9">
-        <f>M369-D369</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O369" t="s">
@@ -16246,7 +16246,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N370" s="9">
-        <f>M370-D370</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O370" t="s">
@@ -16270,7 +16270,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N371" s="9">
-        <f>M371-D371</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O371" t="s">
@@ -16294,7 +16294,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N372" s="9">
-        <f>M372-D372</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O372" t="s">
@@ -16318,7 +16318,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N373" s="9">
-        <f>M373-D373</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O373" t="s">
@@ -16342,7 +16342,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N374" s="9">
-        <f>M374-D374</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O374" t="s">
@@ -16366,7 +16366,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N375" s="9">
-        <f>M375-D375</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O375" t="s">
@@ -16390,7 +16390,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N376" s="9">
-        <f>M376-D376</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O376" t="s">
@@ -16414,7 +16414,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N377" s="9">
-        <f>M377-D377</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O377" t="s">
@@ -16438,7 +16438,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N378" s="9">
-        <f>M378-D378</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O378" t="s">
@@ -16462,7 +16462,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N379" s="9">
-        <f>M379-D379</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O379" t="s">
@@ -16486,7 +16486,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N380" s="9">
-        <f>M380-D380</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O380" t="s">
@@ -16510,7 +16510,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N381" s="9">
-        <f>M381-D381</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O381" t="s">
@@ -16534,7 +16534,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N382" s="9">
-        <f>M382-D382</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O382" t="s">
@@ -16558,7 +16558,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N383" s="9">
-        <f>M383-D383</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O383" t="s">
@@ -16582,7 +16582,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N384" s="9">
-        <f>M384-D384</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O384" t="s">
@@ -16606,7 +16606,7 @@
         <v>0.50902777777777775</v>
       </c>
       <c r="N385" s="9">
-        <f>M385-D385</f>
+        <f t="shared" si="12"/>
         <v>2.5694444444444409E-2</v>
       </c>
       <c r="O385" t="s">
@@ -16630,7 +16630,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N386" s="9">
-        <f>M386-D386</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O386" t="s">
@@ -16654,7 +16654,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N387" s="9">
-        <f>M387-D387</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O387" t="s">
@@ -16678,7 +16678,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N388" s="9">
-        <f>M388-D388</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O388" t="s">
@@ -16702,7 +16702,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N389" s="9">
-        <f>M389-D389</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O389" t="s">
@@ -16726,7 +16726,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N390" s="9">
-        <f>M390-D390</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O390" t="s">
@@ -16750,7 +16750,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N391" s="9">
-        <f>M391-D391</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O391" t="s">
@@ -16774,7 +16774,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N392" s="9">
-        <f>M392-D392</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O392" t="s">
@@ -16798,7 +16798,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N393" s="9">
-        <f>M393-D393</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O393" t="s">
@@ -16822,7 +16822,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N394" s="9">
-        <f>M394-D394</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O394" t="s">
@@ -16846,7 +16846,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N395" s="9">
-        <f>M395-D395</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O395" t="s">
@@ -16870,7 +16870,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N396" s="9">
-        <f>M396-D396</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O396" t="s">
@@ -16896,7 +16896,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N397" s="9">
-        <f>M397-D397</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O397" t="s">
@@ -16922,7 +16922,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N398" s="9">
-        <f>M398-D398</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O398" t="s">
@@ -16948,7 +16948,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N399" s="9">
-        <f>M399-D399</f>
+        <f t="shared" si="12"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O399" t="s">
@@ -16974,7 +16974,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N400" s="9">
-        <f>M400-D400</f>
+        <f t="shared" ref="N400:N431" si="13">M400-D400</f>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O400" t="s">
@@ -17000,7 +17000,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N401" s="9">
-        <f>M401-D401</f>
+        <f t="shared" si="13"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O401" t="s">
@@ -17026,7 +17026,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N402" s="9">
-        <f>M402-D402</f>
+        <f t="shared" si="13"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O402" t="s">
@@ -17052,7 +17052,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N403" s="9">
-        <f>M403-D403</f>
+        <f t="shared" si="13"/>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O403" t="s">
@@ -17078,7 +17078,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N404" s="9">
-        <f>M404-D404</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O404" t="s">
@@ -17104,7 +17104,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N405" s="9">
-        <f>M405-D405</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O405" t="s">
@@ -17130,7 +17130,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N406" s="9">
-        <f>M406-D406</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O406" t="s">
@@ -17156,7 +17156,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N407" s="9">
-        <f>M407-D407</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O407" t="s">
@@ -17182,7 +17182,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N408" s="9">
-        <f>M408-D408</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O408" t="s">
@@ -17208,7 +17208,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N409" s="9">
-        <f>M409-D409</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O409" t="s">
@@ -17234,7 +17234,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N410" s="9">
-        <f>M410-D410</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O410" t="s">
@@ -17260,7 +17260,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N411" s="9">
-        <f>M411-D411</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O411" t="s">
@@ -17286,7 +17286,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N412" s="9">
-        <f>M412-D412</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O412" t="s">
@@ -17312,7 +17312,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N413" s="9">
-        <f>M413-D413</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O413" t="s">
@@ -17338,7 +17338,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N414" s="9">
-        <f>M414-D414</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O414" t="s">
@@ -17364,7 +17364,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N415" s="9">
-        <f>M415-D415</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O415" t="s">
@@ -17390,7 +17390,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N416" s="9">
-        <f>M416-D416</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O416" t="s">
@@ -17416,7 +17416,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N417" s="9">
-        <f>M417-D417</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O417" t="s">
@@ -17442,7 +17442,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N418" s="9">
-        <f>M418-D418</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O418" t="s">
@@ -17468,7 +17468,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N419" s="9">
-        <f>M419-D419</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O419" t="s">
@@ -17494,7 +17494,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N420" s="9">
-        <f>M420-D420</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O420" t="s">
@@ -17520,7 +17520,7 @@
         <v>0.55138888888888893</v>
       </c>
       <c r="N421" s="9">
-        <f>M421-D421</f>
+        <f t="shared" si="13"/>
         <v>1.5972222222222276E-2</v>
       </c>
       <c r="O421" t="s">

</xml_diff>

<commit_message>
secondary figures done. had to fix my messed up D28
</commit_message>
<xml_diff>
--- a/EPFU_2025/EPFU 2025 Bleeding.xlsx
+++ b/EPFU_2025/EPFU 2025 Bleeding.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Ashlyn_thesis\EPFU_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B723B00-76B6-4603-B432-3A737D759798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF270B75-9DCF-4567-8137-4E9501C18E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7726,7 +7726,7 @@
         <v>0.57222222222222219</v>
       </c>
       <c r="N168" s="8">
-        <f t="shared" ref="N168:N199" si="4">M168-D168</f>
+        <f t="shared" ref="N168:N174" si="4">M168-D168</f>
         <v>1.8055555555555491E-2</v>
       </c>
       <c r="O168" t="s">
@@ -12334,7 +12334,7 @@
     </row>
     <row r="272" spans="1:15" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B272" s="4">
         <v>45936</v>
@@ -13681,7 +13681,7 @@
         <v>0.66388888888888886</v>
       </c>
       <c r="N301" s="8">
-        <f t="shared" ref="N301:N332" si="8">M301-D301</f>
+        <f t="shared" ref="N301:N331" si="8">M301-D301</f>
         <v>7.4999999999999956E-2</v>
       </c>
     </row>
@@ -16974,7 +16974,7 @@
         <v>0.5756944444444444</v>
       </c>
       <c r="N400" s="9">
-        <f t="shared" ref="N400:N431" si="13">M400-D400</f>
+        <f t="shared" ref="N400:N421" si="13">M400-D400</f>
         <v>2.0833333333333259E-2</v>
       </c>
       <c r="O400" t="s">

</xml_diff>